<commit_message>
mobile responsiveness, fixed service report, updated tests.
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -6,6 +6,7 @@
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
     <sheet name="Staff" sheetId="2" r:id="rId2"/>
     <sheet name="Ticket" sheetId="3" r:id="rId3"/>
+    <sheet name="ServiceReport" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -551,7 +552,7 @@
         <v/>
       </c>
       <c r="E9">
-        <v>10</v>
+        <v>78787888</v>
       </c>
     </row>
     <row r="10">
@@ -1026,4 +1027,14 @@
     <ignoredError numberStoredAsText="1" sqref="A1:O7"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1"/>
+  <sheetData/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
made slight changes to ticket submission form (no longer requires name for pre-existing customers)
</commit_message>
<xml_diff>
--- a/Database/database.xlsx
+++ b/Database/database.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -589,9 +589,43 @@
         <v>0</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>C-0000000000007</v>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v>the@gaming.thing</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>C-0000000000008</v>
+      </c>
+      <c r="B13" t="str">
+        <v>new name test!!!</v>
+      </c>
+      <c r="C13" t="str">
+        <v>the@gaming.test</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E13"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>